<commit_message>
added parameter values and completed system.py
</commit_message>
<xml_diff>
--- a/qsdsan/data/sanunit_data/VFA/impact_items.xlsx
+++ b/qsdsan/data/sanunit_data/VFA/impact_items.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10102"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10328"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/blues/Documents/QSDsan/qsdsan/data/sanunit_data/VFA/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/blues/Documents/QSDsan/qsdsan/data/sanunit_data/vfa/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{77A90171-2985-0441-A41B-6F23FDECBB13}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{698E7783-B98B-114B-95D1-A46C79F785D6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="760" windowWidth="29400" windowHeight="16760" xr2:uid="{BD97E243-0BB4-3F42-9EBC-00D49E7EE019}"/>
+    <workbookView xWindow="32920" yWindow="-1980" windowWidth="29400" windowHeight="16760" activeTab="1" xr2:uid="{BD97E243-0BB4-3F42-9EBC-00D49E7EE019}"/>
   </bookViews>
   <sheets>
     <sheet name="info" sheetId="2" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="99" uniqueCount="35">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="105" uniqueCount="36">
   <si>
     <t>uniform</t>
   </si>
@@ -140,6 +140,9 @@
   </si>
   <si>
     <t>ea</t>
+  </si>
+  <si>
+    <t>HDPE</t>
   </si>
 </sst>
 </file>
@@ -520,7 +523,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{64D7D79F-DE6E-0748-9640-80C06206B878}">
-  <dimension ref="A1:B15"/>
+  <dimension ref="A1:B16"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.2">
@@ -640,6 +643,14 @@
         <v>30</v>
       </c>
       <c r="B15" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A16" t="s">
+        <v>35</v>
+      </c>
+      <c r="B16" t="s">
         <v>32</v>
       </c>
     </row>
@@ -650,7 +661,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{28627DAA-889C-6942-A3B5-3C8A993554C1}">
-  <dimension ref="A1:J15"/>
+  <dimension ref="A1:J16"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="10.6640625" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="26.6640625" bestFit="1" customWidth="1"/>
@@ -1042,6 +1053,23 @@
         <v>20</v>
       </c>
     </row>
+    <row r="16" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A16" t="s">
+        <v>35</v>
+      </c>
+      <c r="B16" t="s">
+        <v>8</v>
+      </c>
+      <c r="C16">
+        <v>2.75</v>
+      </c>
+      <c r="F16" t="s">
+        <v>0</v>
+      </c>
+      <c r="G16" t="s">
+        <v>20</v>
+      </c>
+    </row>
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>